<commit_message>
fixed artdesign remains problem
</commit_message>
<xml_diff>
--- a/data/ready_stocks/ad-ozon-stocks-updated.xlsx
+++ b/data/ready_stocks/ad-ozon-stocks-updated.xlsx
@@ -536,7 +536,7 @@
         <v/>
       </c>
       <c r="D10">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -550,7 +550,7 @@
         <v/>
       </c>
       <c r="D11">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -578,7 +578,7 @@
         <v/>
       </c>
       <c r="D13">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -690,7 +690,7 @@
         <v/>
       </c>
       <c r="D21">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -788,7 +788,7 @@
         <v/>
       </c>
       <c r="D28">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -802,7 +802,7 @@
         <v/>
       </c>
       <c r="D29">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -886,7 +886,7 @@
         <v/>
       </c>
       <c r="D35">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36">
@@ -998,7 +998,7 @@
         <v/>
       </c>
       <c r="D43">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -1040,7 +1040,7 @@
         <v/>
       </c>
       <c r="D46">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -1222,7 +1222,7 @@
         <v/>
       </c>
       <c r="D59">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -1404,7 +1404,7 @@
         <v/>
       </c>
       <c r="D72">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -1530,7 +1530,7 @@
         <v/>
       </c>
       <c r="D81">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -1852,7 +1852,7 @@
         <v/>
       </c>
       <c r="D104">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -1866,7 +1866,7 @@
         <v/>
       </c>
       <c r="D105">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -1936,7 +1936,7 @@
         <v/>
       </c>
       <c r="D110">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -1964,7 +1964,7 @@
         <v/>
       </c>
       <c r="D112">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="D117">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="118">
@@ -2076,7 +2076,7 @@
         <v/>
       </c>
       <c r="D120">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121">
@@ -2230,7 +2230,7 @@
         <v/>
       </c>
       <c r="D131">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
@@ -2370,7 +2370,7 @@
         <v/>
       </c>
       <c r="D141">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -2412,7 +2412,7 @@
         <v/>
       </c>
       <c r="D144">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
@@ -2440,7 +2440,7 @@
         <v/>
       </c>
       <c r="D146">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147">
@@ -2468,7 +2468,7 @@
         <v/>
       </c>
       <c r="D148">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149">
@@ -2538,7 +2538,7 @@
         <v/>
       </c>
       <c r="D153">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154">
@@ -2552,7 +2552,7 @@
         <v/>
       </c>
       <c r="D154">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>